<commit_message>
-Updated Public dungeon mapId -Updated zone names but PTS is still missing lots of translations :-(
</commit_message>
<xml_diff>
--- a/LibZone/LibZone_Maps.xlsx
+++ b/LibZone/LibZone_Maps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pzieg\Documents\Elder Scrolls Online\pts\AddOns\LibZone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD096FD2-0650-4909-A35B-8AB5C3AC9E19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F44870-EAB1-45E9-B920-1BFD774F68A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2073" uniqueCount="1312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2079" uniqueCount="1316">
   <si>
     <t>Glenumbra</t>
   </si>
@@ -3975,6 +3975,18 @@
   </si>
   <si>
     <t xml:space="preserve">Silorn </t>
+  </si>
+  <si>
+    <t>Calindvale Gardens</t>
+  </si>
+  <si>
+    <t>Calindvale Gärten</t>
+  </si>
+  <si>
+    <t>Sonnenwende</t>
+  </si>
+  <si>
+    <t>Solstice</t>
   </si>
 </sst>
 </file>
@@ -4055,7 +4067,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -4076,6 +4088,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -4358,7 +4373,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:D1879"/>
+  <dimension ref="A1:D1880"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="47.5703125" bestFit="1" customWidth="1"/>
@@ -34392,10 +34407,10 @@
       </c>
     </row>
     <row r="1878" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1878" s="9">
+      <c r="A1878">
         <v>2456</v>
       </c>
-      <c r="B1878" s="9" t="s">
+      <c r="B1878" t="s">
         <v>1308</v>
       </c>
       <c r="C1878" s="6" t="s">
@@ -34407,18 +34422,33 @@
       </c>
     </row>
     <row r="1879" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1879" s="9">
+      <c r="A1879">
         <v>2441</v>
       </c>
-      <c r="B1879" s="9" t="s">
+      <c r="B1879" t="s">
         <v>1311</v>
       </c>
       <c r="C1879" s="6" t="s">
         <v>1296</v>
       </c>
       <c r="D1879" s="7" t="str">
-        <f t="shared" ref="D1879" si="31">IF(C1879="X","["&amp;A1879&amp;"]=true,     --"&amp;B1879,"")</f>
+        <f t="shared" ref="D1879:D1880" si="31">IF(C1879="X","["&amp;A1879&amp;"]=true,     --"&amp;B1879,"")</f>
         <v xml:space="preserve">[2441]=true,     --Silorn </v>
+      </c>
+    </row>
+    <row r="1880" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1880" s="10">
+        <v>2728</v>
+      </c>
+      <c r="B1880" s="9" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C1880" s="6" t="s">
+        <v>1296</v>
+      </c>
+      <c r="D1880" s="7" t="str">
+        <f t="shared" si="31"/>
+        <v>[2728]=true,     --Calindvale Gardens</v>
       </c>
     </row>
   </sheetData>
@@ -34444,7 +34474,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{189622CA-1B52-4A0C-9E87-D4E1EF536BE4}">
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.5703125" bestFit="1" customWidth="1"/>
@@ -35071,31 +35101,45 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="9" t="s">
+      <c r="A45" s="8" t="s">
         <v>1310</v>
       </c>
-      <c r="B45" s="9" t="s">
+      <c r="B45" s="8" t="s">
         <v>1308</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="8" t="s">
         <v>1306</v>
       </c>
-      <c r="D45" s="9" t="s">
+      <c r="D45" s="8" t="s">
         <v>1307</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="9" t="s">
+      <c r="A46" s="8" t="s">
         <v>1309</v>
       </c>
-      <c r="B46" s="9" t="s">
+      <c r="B46" s="8" t="s">
         <v>1309</v>
       </c>
-      <c r="C46" s="9" t="s">
+      <c r="C46" s="8" t="s">
         <v>1306</v>
       </c>
-      <c r="D46" s="9" t="s">
+      <c r="D46" s="8" t="s">
         <v>1307</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="9" t="s">
+        <v>1313</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>1314</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>1315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>